<commit_message>
hapus package lock json
</commit_message>
<xml_diff>
--- a/avatar-apbd/excel/realisasi/dtrealtest1.xlsx
+++ b/avatar-apbd/excel/realisasi/dtrealtest1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\AVATARAPBD\avatar-apbd\excel\realisasi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{81B9E571-E78C-44B1-9C7C-E97595D096B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F371A60-BF9D-421C-AC52-6A217F1D5F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{698132E3-C4E2-41ED-8FF1-EFA227F35D0F}"/>
   </bookViews>
@@ -1616,10 +1616,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{110E5EC8-6D3C-42E0-BA64-608AB1A2C1BE}">
-  <dimension ref="A1:K713"/>
+  <dimension ref="A1:O713"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="12" max="12" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>396</v>
       </c>
@@ -1654,7 +1658,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>407</v>
       </c>
@@ -1688,8 +1692,15 @@
       <c r="K2">
         <v>1250000</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L2">
+        <f>SUM(J2:J713)</f>
+        <v>228468183128.85001</v>
+      </c>
+      <c r="O2">
+        <v>96728954071</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>407</v>
       </c>
@@ -1723,8 +1734,11 @@
       <c r="K3">
         <v>3585000</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="O3">
+        <v>146353889743</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>407</v>
       </c>
@@ -1758,8 +1772,12 @@
       <c r="K4">
         <v>95165000</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="O4">
+        <f>(O2/O3)*100</f>
+        <v>66.092506486064522</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>407</v>
       </c>
@@ -1793,8 +1811,12 @@
       <c r="K5">
         <v>2069501.5</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="O5">
+        <f>(O3/O2)*100</f>
+        <v>151.30308308262573</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>407</v>
       </c>
@@ -1829,7 +1851,7 @@
         <v>1390500</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>407</v>
       </c>
@@ -1864,7 +1886,7 @@
         <v>2830350</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>407</v>
       </c>
@@ -1899,7 +1921,7 @@
         <v>15000000</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>407</v>
       </c>
@@ -1934,7 +1956,7 @@
         <v>22499998.5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>407</v>
       </c>
@@ -1969,7 +1991,7 @@
         <v>38103750</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>407</v>
       </c>
@@ -2004,7 +2026,7 @@
         <v>6300000</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>407</v>
       </c>
@@ -2039,7 +2061,7 @@
         <v>127500000</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>407</v>
       </c>
@@ -2074,7 +2096,7 @@
         <v>135000000</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>407</v>
       </c>
@@ -2109,7 +2131,7 @@
         <v>1249000.01</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>407</v>
       </c>
@@ -2144,7 +2166,7 @@
         <v>2184000</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>407</v>
       </c>

</xml_diff>